<commit_message>
fix: recognise distributor maker spellings; sample Read me reflects live data
Nexperia USA Inc., Panasonic Industry, TE Connectivity ALCOSWITCH Switches and
similar names now match the BOM's maker, so live data no longer raises false
'Manufacturer differs' warnings.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/samples/QuoteLens-sample-BOM.xlsx
+++ b/apps/web/public/samples/QuoteLens-sample-BOM.xlsx
@@ -2968,7 +2968,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>3 blockers stop the quote. Every risk explains why, with evidence.</t>
+          <t>Blockers stop the quote (F1 and J2 always; obsolete parts depend on the market). Every risk explains why, with evidence.</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>F1: enter a part number. J2: correct the quantity. Hall sensor U11-U13: Find alternates and approve the drop-in.</t>
+          <t>F1: enter a part number. J2: correct the quantity. An obsolete part: Find alternates and approve a drop-in, or waive it with a reason.</t>
         </is>
       </c>
     </row>
@@ -3035,7 +3035,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Prices, stock and lifecycle come from the QuoteLens demo catalog (synthetic values).</t>
+          <t>Prices, stock and lifecycle are fetched live from DigiKey, Mouser and element14, so remarks about the market may differ from today's data.</t>
         </is>
       </c>
       <c r="B15" s="4" t="n"/>

</xml_diff>